<commit_message>
feat: se ha implementado la funcionalidad de que se pueda cambiar el excel en tiempo de ejecucion
se ha implementado gracias a watchlife un Simple, modern and high performance file watching and code reload in python. la visualización del documento excel que contiene a los alumnos permitidos para utilizar el agente docente.

Además se ha implementado una nueva tabla en la base de datos para poder tenerlos guardados en una base de datos y consultarlo en la bbdd y no directamente en el excel
</commit_message>
<xml_diff>
--- a/code/data/alumnos_autorizados.xlsx
+++ b/code/data/alumnos_autorizados.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\Multi-Agent-Programming-Teacher\code\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D62FBE-3A53-4E5F-BC38-813834FEB8EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3D9A39B-DD2F-4211-818F-DB85F0706AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{193370B4-417B-4FA5-9C95-ABB2EF3461F7}"/>
+    <workbookView xWindow="4020" yWindow="3015" windowWidth="21600" windowHeight="11295" xr2:uid="{193370B4-417B-4FA5-9C95-ABB2EF3461F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,17 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Nombre</t>
   </si>
   <si>
-    <t>Curso</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
     <t xml:space="preserve">alejandro </t>
   </si>
   <si>
@@ -57,6 +51,39 @@
   </si>
   <si>
     <t>estefania@um.es</t>
+  </si>
+  <si>
+    <t>DNI</t>
+  </si>
+  <si>
+    <t>ala</t>
+  </si>
+  <si>
+    <t>juan@um.es</t>
+  </si>
+  <si>
+    <t>233456563K</t>
+  </si>
+  <si>
+    <t>444422244P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">juan </t>
+  </si>
+  <si>
+    <t>jjuuuaaann@um.es</t>
+  </si>
+  <si>
+    <t>3332211122P</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>a@um.es</t>
+  </si>
+  <si>
+    <t>Correo electrónico</t>
   </si>
 </sst>
 </file>
@@ -439,7 +466,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BDE2F41-FD62-496E-9627-833238572546}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -447,43 +474,73 @@
     <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B2">
+      <c r="B3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{0F24FA43-8FDE-4003-8532-3E654F883707}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{987D857F-90D5-48AD-9C77-8D5AFFD9A06D}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{0F24FA43-8FDE-4003-8532-3E654F883707}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{987D857F-90D5-48AD-9C77-8D5AFFD9A06D}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{7649F954-6CD5-4F97-8F69-70F5CE42D5D9}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{20BD5D74-92D3-4C6E-91AD-5ED66C8D7BC0}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{9BB7C650-A564-4AC3-9650-AA01D2DFD598}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implementados con exito el inicio de sesion y el registrar usuario en la web
</commit_message>
<xml_diff>
--- a/code/data/alumnos_autorizados.xlsx
+++ b/code/data/alumnos_autorizados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\Multi-Agent-Programming-Teacher\code\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3D9A39B-DD2F-4211-818F-DB85F0706AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AD12A2C-C81A-43FB-9598-58B7B268D39D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4020" yWindow="3015" windowWidth="21600" windowHeight="11295" xr2:uid="{193370B4-417B-4FA5-9C95-ABB2EF3461F7}"/>
+    <workbookView xWindow="4365" yWindow="3360" windowWidth="21600" windowHeight="11295" xr2:uid="{193370B4-417B-4FA5-9C95-ABB2EF3461F7}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Nombre</t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>Correo electrónico</t>
+  </si>
+  <si>
+    <t>prueba</t>
+  </si>
+  <si>
+    <t>prueba@um.es</t>
   </si>
 </sst>
 </file>
@@ -466,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BDE2F41-FD62-496E-9627-833238572546}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -534,6 +540,14 @@
         <v>14</v>
       </c>
     </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{0F24FA43-8FDE-4003-8532-3E654F883707}"/>
@@ -541,6 +555,7 @@
     <hyperlink ref="B4" r:id="rId3" xr:uid="{7649F954-6CD5-4F97-8F69-70F5CE42D5D9}"/>
     <hyperlink ref="B5" r:id="rId4" xr:uid="{20BD5D74-92D3-4C6E-91AD-5ED66C8D7BC0}"/>
     <hyperlink ref="B6" r:id="rId5" xr:uid="{9BB7C650-A564-4AC3-9650-AA01D2DFD598}"/>
+    <hyperlink ref="B7" r:id="rId6" xr:uid="{32DAA6AF-7B72-4541-941C-54759A491593}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: errores que hacian que el agente docente se quedara pillado o no hiciese bien las cosas
</commit_message>
<xml_diff>
--- a/code/data/alumnos_autorizados.xlsx
+++ b/code/data/alumnos_autorizados.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\Multi-Agent-Programming-Teacher\code\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D86A1CD4-78BD-477B-8CED-946B6A6AB986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292251AE-301F-4CB4-8EE7-9A68930AC278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4365" yWindow="3360" windowWidth="21600" windowHeight="11295" xr2:uid="{193370B4-417B-4FA5-9C95-ABB2EF3461F7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Nombre</t>
   </si>
@@ -96,6 +96,12 @@
   </si>
   <si>
     <t>olga@um.es</t>
+  </si>
+  <si>
+    <t>aa</t>
+  </si>
+  <si>
+    <t>aa@um.es</t>
   </si>
 </sst>
 </file>
@@ -487,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BDE2F41-FD62-496E-9627-833238572546}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -572,6 +578,14 @@
       </c>
       <c r="D8" s="2"/>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{0F24FA43-8FDE-4003-8532-3E654F883707}"/>
@@ -581,6 +595,7 @@
     <hyperlink ref="B6" r:id="rId5" xr:uid="{9BB7C650-A564-4AC3-9650-AA01D2DFD598}"/>
     <hyperlink ref="B7" r:id="rId6" xr:uid="{32DAA6AF-7B72-4541-941C-54759A491593}"/>
     <hyperlink ref="B8" r:id="rId7" xr:uid="{6998089D-D6E6-41F6-89D2-6E91AD4173DE}"/>
+    <hyperlink ref="B9" r:id="rId8" xr:uid="{E2EE4D06-3560-4958-A727-8AFB4A767F76}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>